<commit_message>
improved test skipping logic with descriptive skip messages
</commit_message>
<xml_diff>
--- a/test-data/login_data.xlsx
+++ b/test-data/login_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/4c11ee890eb53755/Documents/Testing/Playwright_TypeScript/test-data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_BB7CC0C09EFCB6DB99C23934A309CAF48AA51E01" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F7FA9E71-2AA8-4896-9540-8B758BF71942}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="11_BB7CC0C09EFCB6DB99C23934A309CAF48AA51E01" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F92C42FC-DABE-416B-BCB9-B1021F521E24}"/>
   <bookViews>
     <workbookView xWindow="13170" yWindow="680" windowWidth="20790" windowHeight="18670" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="12">
   <si>
     <t>username</t>
   </si>
@@ -58,6 +58,9 @@
   </si>
   <si>
     <t>problem_user</t>
+  </si>
+  <si>
+    <t>no</t>
   </si>
 </sst>
 </file>
@@ -126,6 +129,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
   <a:themeElements>
@@ -281,7 +288,7 @@
         <v>9</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4" spans="1:4" ht="13" x14ac:dyDescent="0.3">
@@ -295,7 +302,7 @@
         <v>6</v>
       </c>
       <c r="D4" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
     </row>
   </sheetData>

</xml_diff>